<commit_message>
Retire la fiche de test du pipeline
</commit_message>
<xml_diff>
--- a/data/frise-philosophes-greco-romains.xlsx
+++ b/data/frise-philosophes-greco-romains.xlsx
@@ -571,7 +571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:M101"/>
+  <dimension ref="A1:M100"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="6.39" customWidth="1" style="19" min="1" max="2"/>
@@ -6727,29 +6727,7 @@
         </is>
       </c>
     </row>
-    <row r="101" ht="15" customHeight="1" s="21">
-      <c r="A101" t="n">
-        <v>-350</v>
-      </c>
-      <c r="B101" t="n">
-        <v>-280</v>
-      </c>
-      <c r="C101" t="inlineStr">
-        <is>
-          <t>- 350 A JC  - 280 A JC</t>
-        </is>
-      </c>
-      <c r="D101" t="inlineStr">
-        <is>
-          <t>TESTUS Philosophus</t>
-        </is>
-      </c>
-      <c r="E101" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Fiche de test pour valider le bat.&lt;/p&gt;</t>
-        </is>
-      </c>
-    </row>
+    <row r="101" ht="15" customHeight="1" s="21"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
Demo complete: fiche + portrait
</commit_message>
<xml_diff>
--- a/data/frise-philosophes-greco-romains.xlsx
+++ b/data/frise-philosophes-greco-romains.xlsx
@@ -571,7 +571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:M100"/>
+  <dimension ref="A1:M101"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="6.39" customWidth="1" style="19" min="1" max="2"/>
@@ -6727,7 +6727,34 @@
         </is>
       </c>
     </row>
-    <row r="101" ht="15" customHeight="1" s="21"/>
+    <row r="101" ht="15" customHeight="1" s="21">
+      <c r="A101" t="n">
+        <v>-350</v>
+      </c>
+      <c r="B101" t="n">
+        <v>-280</v>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>- 350 A JC  - 280 A JC</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>DEMO Test Philosophe</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Fiche de demonstration complete (xlsx + portrait).&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>/pho/demo-test-philosophe-mini.webp</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
Retire la demo complete
</commit_message>
<xml_diff>
--- a/data/frise-philosophes-greco-romains.xlsx
+++ b/data/frise-philosophes-greco-romains.xlsx
@@ -571,7 +571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:M101"/>
+  <dimension ref="A1:M100"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="6.39" customWidth="1" style="19" min="1" max="2"/>
@@ -6727,34 +6727,7 @@
         </is>
       </c>
     </row>
-    <row r="101" ht="15" customHeight="1" s="21">
-      <c r="A101" t="n">
-        <v>-350</v>
-      </c>
-      <c r="B101" t="n">
-        <v>-280</v>
-      </c>
-      <c r="C101" t="inlineStr">
-        <is>
-          <t>- 350 A JC  - 280 A JC</t>
-        </is>
-      </c>
-      <c r="D101" t="inlineStr">
-        <is>
-          <t>DEMO Test Philosophe</t>
-        </is>
-      </c>
-      <c r="E101" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Fiche de demonstration complete (xlsx + portrait).&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="H101" t="inlineStr">
-        <is>
-          <t>/pho/demo-test-philosophe-mini.webp</t>
-        </is>
-      </c>
-    </row>
+    <row r="101" ht="15" customHeight="1" s="21"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
Corrige les 29 points signalés par la vérification des données
- Courant « Constructivisme (politique) » renommé « Constructivisme »,
  lien Wikipédia vers Constructivisme (épistémologie) : les 23 fiches qui
  y renvoyaient (Kant, Bachelard, Kuhn, Latour…) affichent de nouveau le
  lien. Redirection inversée.
- « Comptabilisme » corrigé en « Compatibilisme » (courant et fiche de
  Chrysippe) ; Hobbes y est désormais rattaché. Redirection 301.
- Dates vérifiées sur Wikipédia : Héraclite, Gorgias, Boèce, Alexandre de
  Halès, Lorenzo Valla, Hubert Damisch, Tran Duc Thao.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-philosophes-greco-romains.xlsx
+++ b/data/frise-philosophes-greco-romains.xlsx
@@ -1139,7 +1139,7 @@
       </c>
       <c r="C11" s="27" t="inlineStr">
         <is>
-          <t xml:space="preserve"> - 576 A JC  - 480 A JC  </t>
+          <t xml:space="preserve"> - 535 A JC  - 480 A JC  </t>
         </is>
       </c>
       <c r="D11" s="28" t="inlineStr">
@@ -1520,7 +1520,7 @@
       </c>
       <c r="C17" s="27" t="inlineStr">
         <is>
-          <t>-480 AJC   - 356 AJC</t>
+          <t xml:space="preserve">-480 AJC   - 375 AJC</t>
         </is>
       </c>
       <c r="D17" s="28" t="inlineStr">
@@ -3690,7 +3690,7 @@
       </c>
       <c r="L51" s="21" t="inlineStr">
         <is>
-          <t>Stoïcisme ; Déterminisme ; Comptabilisme</t>
+          <t xml:space="preserve">Stoïcisme ; Déterminisme ; Compatibilisme</t>
         </is>
       </c>
       <c r="M51" s="21" t="inlineStr">
@@ -6207,8 +6207,8 @@
       </c>
     </row>
     <row r="92" ht="136.5" customHeight="1" s="22">
-      <c r="A92" s="27" t="n">
-        <v>472</v>
+      <c r="A92" s="27">
+        <v>480</v>
       </c>
       <c r="B92" s="27" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fiches — 24 fiches nouvelles : ATHANASE d'Alexandrie, JEAN CHRYSOSTOME, HIPPOLYTE de Rome, ASPASIE de Milet, BARLAAM de Calabre, Ludwig von MISES et 18 autre(s)
Publié depuis l'éditeur des fiches.
</commit_message>
<xml_diff>
--- a/data/frise-philosophes-greco-romains.xlsx
+++ b/data/frise-philosophes-greco-romains.xlsx
@@ -3227,7 +3227,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:P119"/>
+  <dimension ref="A1:P123"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="1" width="6.39"/>
@@ -9078,6 +9078,239 @@
         </is>
       </c>
       <c r="P119"/>
+    </row>
+    <row r="120" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A120" s="7">
+        <v>298</v>
+      </c>
+      <c r="B120" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">373</t>
+        </is>
+      </c>
+      <c r="C120" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vers 298 – 373</t>
+        </is>
+      </c>
+      <c r="D120" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ATHANASE d'Alexandrie</t>
+        </is>
+      </c>
+      <c r="E120" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Athanase_d%27Alexandrie" title=" Wikipedia"&gt;ATHANASE d'Alexandrie&lt;/a&gt; est un évêque et théologien chrétien de langue grecque. Né vers 298 à Alexandrie, en Égypte, il est encore jeune diacre quand il accompagne son évêque au concile de Nicée, en 325. Le concile condamne alors Arius, un prêtre alexandrin qui enseignait que le Fils de Dieu n’est pas éternel, mais créé par le Père. Devenu évêque d’Alexandrie en 328, Athanase consacre toute sa vie à défendre la foi de Nicée : le Fils est « de même substance » que le Père, pleinement Dieu comme lui.&lt;/p&gt; &lt;p&gt;Ce combat lui vaut l’hostilité de plusieurs empereurs, favorables aux ariens. Il est exilé cinq fois, notamment à Trèves, en Gaule, et passe au total dix-sept ans loin de son siège, parfois caché chez les moines du désert. On a dit de lui qu’il était seul contre le monde. Dans &lt;em&gt;Sur l’incarnation du Verbe&lt;/em&gt;, il explique pourquoi le Christ doit être vraiment Dieu : seul Dieu peut sauver l’homme de la mort et le transformer. Sa formule est restée célèbre : « Dieu s’est fait homme pour que l’homme devienne Dieu. »&lt;/p&gt; &lt;p&gt;Sa &lt;em&gt;Vie d’Antoine&lt;/em&gt;, consacrée au père des moines d’Égypte, fait connaître le monachisme dans tout le monde chrétien et devient le modèle des vies de saints. Augustin raconte, dans ses &lt;em&gt;Confessions&lt;/em&gt;, l’effet que sa lecture produisit sur lui et ses amis. En 367, une de ses lettres donne pour la première fois la liste exacte des vingt-sept livres du Nouveau Testament. Il meurt à Alexandrie en 373. Il est une grande figure de la &lt;a href="https://fr.wikipedia.org/wiki/Patristique" title=" Wikipedia"&gt;patristique&lt;/a&gt;.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="H120" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/athanase-mini.webp</t>
+        </is>
+      </c>
+      <c r="J120" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Égyptienne</t>
+        </is>
+      </c>
+      <c r="K120" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">spiritualite ; metaphysique</t>
+        </is>
+      </c>
+      <c r="L120" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Patristique</t>
+        </is>
+      </c>
+      <c r="M120" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">évêque d’Alexandrie, défenseur infatigable de la divinité du Christ contre Arius, auteur de la Vie d’Antoine.</t>
+        </is>
+      </c>
+      <c r="O120" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="P120">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="121" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A121" s="7">
+        <v>349</v>
+      </c>
+      <c r="B121" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">407</t>
+        </is>
+      </c>
+      <c r="C121" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vers 349 – 407</t>
+        </is>
+      </c>
+      <c r="D121" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">JEAN CHRYSOSTOME</t>
+        </is>
+      </c>
+      <c r="E121" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Jean_Chrysostome" title=" Wikipedia"&gt;JEAN CHRYSOSTOME&lt;/a&gt; est un prêtre, archevêque et théologien chrétien de langue grecque, le plus célèbre prédicateur de l’Église ancienne. Né vers 349 à Antioche, en Syrie, il étudie la rhétorique auprès du grand orateur païen Libanios, puis mène plusieurs années une vie d’ermite si rude qu’elle ruine sa santé. Ordonné prêtre à Antioche, il y prêche pendant douze ans devant des foules immenses. Son éloquence lui vaudra, après sa mort, le surnom de « Chrysostome », c’est-à-dire « Bouche d’or ».&lt;/p&gt; &lt;p&gt;Ses centaines d’homélies commentent la Bible verset par verset, surtout l’Évangile de Matthieu et les lettres de saint Paul, en tirant des leçons pour la vie quotidienne. Il y insiste sur la justice sociale : les biens de la terre appartiennent à tous, et le riche n’en est que l’intendant ; refuser de partager, c’est voler les pauvres. Il demande aux chrétiens de reconnaître le Christ dans le mendiant. Ses sermons contiennent aussi des attaques violentes contre les juifs, qui ont pesé lourd dans l’histoire de l’antijudaïsme chrétien.&lt;/p&gt; &lt;p&gt;En 398, il devient archevêque de Constantinople. Il réforme le clergé, réduit le train de vie de l’Église et critique le luxe de la cour, ce qui l’oppose à l’impératrice Eudoxie. Déposé par un synode, il est exilé en Arménie et meurt en 407, épuisé par une marche forcée. La liturgie la plus célébrée dans les Églises orthodoxes porte son nom. Il est l’un des grands noms de la &lt;a href="https://fr.wikipedia.org/wiki/Patristique" title=" Wikipedia"&gt;patristique&lt;/a&gt;.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="H121" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/chrysostome-mini.webp</t>
+        </is>
+      </c>
+      <c r="J121" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Syrienne</t>
+        </is>
+      </c>
+      <c r="K121" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">spiritualite ; ethique</t>
+        </is>
+      </c>
+      <c r="L121" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Patristique</t>
+        </is>
+      </c>
+      <c r="M121" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Père de l’Église grec, prédicateur surnommé « Bouche d’or », archevêque de Constantinople mort en exil.</t>
+        </is>
+      </c>
+      <c r="O121" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="P121">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="122" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A122" s="7">
+        <v>170</v>
+      </c>
+      <c r="B122" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">235</t>
+        </is>
+      </c>
+      <c r="C122" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vers 170 – vers 235</t>
+        </is>
+      </c>
+      <c r="D122" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HIPPOLYTE de Rome</t>
+        </is>
+      </c>
+      <c r="E122" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Hippolyte_de_Rome" title=" Wikipedia"&gt;HIPPOLYTE de Rome&lt;/a&gt; est un prêtre et théologien chrétien de langue grecque, qui vécut à Rome. Né vers 170, peut-être en Orient, il devient l’une des grandes figures de l’Église de Rome au début du IIIe siècle. Exigeant et rigoureux, il s’oppose aux papes Zéphyrin et Calliste, qu’il juge trop indulgents envers les pécheurs et trop vagues sur la distinction entre le Père et le Fils. Il se sépare d’eux et prend la tête d’une communauté dissidente : on le considère parfois comme le premier antipape.&lt;/p&gt; &lt;p&gt;Son œuvre principale, la &lt;em&gt;Réfutation de toutes les hérésies&lt;/em&gt;, a été redécouverte au XIXe siècle dans un monastère du mont Athos. Pour lui, les hérésies chrétiennes ne viennent pas de l’Écriture, mais de la philosophie grecque, des mystères païens et de l’astrologie. Pour le montrer, il consacre son premier livre à un résumé des doctrines des philosophes grecs, de Thalès à Épicure. Ce tableau et les citations qu’il contient, notamment de nombreux fragments d’Héraclite, sont une source précieuse pour connaître la pensée des premiers philosophes.&lt;/p&gt; &lt;p&gt;On lui a longtemps attribué la &lt;em&gt;Tradition apostolique&lt;/em&gt;, qui décrit l’organisation et la liturgie de l’Église ancienne, mais cette attribution est aujourd’hui discutée. En 235, il est déporté dans les mines de Sardaigne avec le pape Pontien, se réconcilie avec lui et y meurt. Il est honoré comme saint et martyr. Il appartient à la &lt;a href="https://fr.wikipedia.org/wiki/Patristique" title=" Wikipedia"&gt;patristique&lt;/a&gt;.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="H122" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/hippolyte-mini.webp</t>
+        </is>
+      </c>
+      <c r="J122" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Romaine</t>
+        </is>
+      </c>
+      <c r="K122" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">spiritualite ; metaphysique</t>
+        </is>
+      </c>
+      <c r="L122" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Patristique</t>
+        </is>
+      </c>
+      <c r="M122" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">prêtre et théologien de Rome, auteur de la Réfutation de toutes les hérésies, précieuse source sur les philosophes grecs.</t>
+        </is>
+      </c>
+      <c r="O122" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="P122"/>
+    </row>
+    <row r="123" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A123" s="7">
+        <v>-470</v>
+      </c>
+      <c r="B123" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-400</t>
+        </is>
+      </c>
+      <c r="C123" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ve siècle A JC</t>
+        </is>
+      </c>
+      <c r="D123" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ASPASIE de Milet</t>
+        </is>
+      </c>
+      <c r="E123" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Aspasie" title=" Wikipedia"&gt;ASPASIE de Milet&lt;/a&gt; est une femme de l’Athènes classique, célèbre pour son intelligence et son art de la parole. Née vers 470 avant notre ère à Milet, une cité grecque d’Asie Mineure, elle s’installe à Athènes, où elle devient la compagne de Périclès, le grand homme d’État de la cité. Étrangère, elle ne peut l’épouser légalement, mais elle lui donne un fils. Sa liberté, sa culture et son influence choquent : les poètes comiques la présentent comme une courtisane qui mènerait Périclès, et on l’accuse même d’impiété. On ignore la date de sa mort.&lt;/p&gt; &lt;p&gt;Les témoignages sur sa pensée viennent surtout des disciples de Socrate, ce qui montre l’estime dont elle jouissait dans ce cercle. Dans le &lt;em&gt;Ménexène&lt;/em&gt; de Platon, Socrate prétend réciter un discours funèbre en l’honneur des Athéniens morts à la guerre, qu’Aspasie lui aurait appris ; il affirme même qu’elle aurait écrit celui, si célèbre, de Périclès. Chez Xénophon, Socrate la recommande comme la meilleure conseillère sur le mariage et la vie du couple.&lt;/p&gt; &lt;p&gt;Un dialogue perdu d’Eschine, un autre disciple de Socrate, la montrait interrogeant un couple : chacun préférerait-il les biens les plus beaux, l’or, les vêtements, puis l’époux le meilleur ? Ce raisonnement, qui part d’exemples pour arriver à une conclusion générale, est cité par Cicéron comme un modèle d’induction. Il est difficile de distinguer la femme réelle de la légende, mais elle reste une figure de la femme philosophe dans l’Antiquité, proche du &lt;a href="https://fr.wikipedia.org/wiki/Socrate" title=" Wikipedia"&gt;cercle de Socrate&lt;/a&gt;.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="H123" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/aspasie-mini.webp</t>
+        </is>
+      </c>
+      <c r="J123" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Grecque</t>
+        </is>
+      </c>
+      <c r="K123" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">politique ; langage</t>
+        </is>
+      </c>
+      <c r="L123" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Socratisme ; Sophisme</t>
+        </is>
+      </c>
+      <c r="M123" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">femme cultivée de l’Athènes de Périclès, que Socrate disait son maître en éloquence.</t>
+        </is>
+      </c>
+      <c r="N123" t="inlineStr">
+        <is>
+          <t xml:space="preserve">femme</t>
+        </is>
+      </c>
+      <c r="O123" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="P123"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>